<commit_message>
updated all files - news added
</commit_message>
<xml_diff>
--- a/individual_details.xlsx
+++ b/individual_details.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\css6\Dropbox\A\ASQ\sutherlandecology\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18A173C8-CCC3-4D81-9EA7-9C2ACD463C07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F012FEE8-8C78-4E26-AA92-E83A39CD3A73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{DEC350D0-BA79-4816-9F19-79808F91A9D5}"/>
   </bookViews>
@@ -19,7 +19,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$O$10</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="157">
   <si>
     <t>Name</t>
   </si>
@@ -450,9 +449,6 @@
     <t>Spatial population ecology of the Diamondback Terrapin at their northern range limit</t>
   </si>
   <si>
-    <t>How do recreational activities alter spatiotemporal species interactions networks, and can this knowledge assist in promoting pro-environmental behaviour?</t>
-  </si>
-  <si>
     <t>Senior Lecturer, Harper Adams University</t>
   </si>
   <si>
@@ -505,6 +501,36 @@
   </si>
   <si>
     <t>https://www.linkedin.com/in/rekha-mohan-239492319/</t>
+  </si>
+  <si>
+    <t>cowans.jpg</t>
+  </si>
+  <si>
+    <t>How can conservation technology advance our understanding of recreational disturbance effects on wildlife, and how can pro-environmental behaviour be encouraged in outdoor recreationists?</t>
+  </si>
+  <si>
+    <t>https://www.linkedin.com/in/amber-cowans/</t>
+  </si>
+  <si>
+    <t>https://ac-ecology.github.io/amber-cowans.website/</t>
+  </si>
+  <si>
+    <t>https://x.com/AmberCowans</t>
+  </si>
+  <si>
+    <t>Gonçalo Curveira-Santos</t>
+  </si>
+  <si>
+    <t>Researcher, CIBIO (Research Centre in Biodiversity and Genetic Resources)</t>
+  </si>
+  <si>
+    <t>Responses of carnivore assemblages to conservation and management models in South Africa</t>
+  </si>
+  <si>
+    <t>https://www.cibio.up.pt/en/people/details/goncalo-curveira-santos/details/</t>
+  </si>
+  <si>
+    <t>https://www.researchgate.net/profile/Goncalo-Curveira-Santos</t>
   </si>
 </sst>
 </file>
@@ -924,15 +950,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{562D1C5D-4376-4368-B05B-B138A3256B7B}">
-  <dimension ref="A1:O32"/>
+  <dimension ref="A1:O33"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="21.36328125" customWidth="1"/>
+    <col min="1" max="1" width="21.453125" customWidth="1"/>
     <col min="2" max="2" width="9" customWidth="1"/>
     <col min="3" max="3" width="18.7265625" customWidth="1"/>
     <col min="4" max="4" width="14.453125" customWidth="1"/>
     <col min="5" max="5" width="10.81640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="12.08984375" customWidth="1"/>
+    <col min="8" max="8" width="12.1796875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:15" x14ac:dyDescent="0.35">
@@ -1134,7 +1160,7 @@
         <v>37</v>
       </c>
       <c r="O5" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="6" spans="1:15" x14ac:dyDescent="0.35">
@@ -1221,10 +1247,10 @@
         <v>14</v>
       </c>
       <c r="H8" t="s">
+        <v>145</v>
+      </c>
+      <c r="J8" t="s">
         <v>146</v>
-      </c>
-      <c r="J8" t="s">
-        <v>147</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.35">
@@ -1238,19 +1264,28 @@
         <v>113</v>
       </c>
       <c r="D9" t="s">
-        <v>19</v>
+        <v>147</v>
       </c>
       <c r="E9" t="s">
         <v>13</v>
       </c>
       <c r="F9">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="G9" t="s">
         <v>14</v>
       </c>
       <c r="H9" t="s">
-        <v>129</v>
+        <v>148</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="M9" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.35">
@@ -1482,7 +1517,7 @@
         <v>113</v>
       </c>
       <c r="D17" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E17" t="s">
         <v>13</v>
@@ -1494,10 +1529,10 @@
         <v>14</v>
       </c>
       <c r="H17" t="s">
+        <v>131</v>
+      </c>
+      <c r="J17" s="2" t="s">
         <v>132</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.35">
@@ -1534,7 +1569,7 @@
         <v>113</v>
       </c>
       <c r="D19" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E19" t="s">
         <v>13</v>
@@ -1546,10 +1581,10 @@
         <v>14</v>
       </c>
       <c r="H19" t="s">
+        <v>137</v>
+      </c>
+      <c r="J19" s="2" t="s">
         <v>138</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="20" spans="1:12" x14ac:dyDescent="0.35">
@@ -1747,7 +1782,7 @@
         <v>1</v>
       </c>
       <c r="C28" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D28" t="s">
         <v>19</v>
@@ -1770,13 +1805,13 @@
     </row>
     <row r="29" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B29">
         <v>1</v>
       </c>
       <c r="C29" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D29" t="s">
         <v>19</v>
@@ -1854,16 +1889,16 @@
     </row>
     <row r="32" spans="1:12" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B32">
         <v>1</v>
       </c>
       <c r="C32" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="D32" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E32" t="s">
         <v>13</v>
@@ -1875,13 +1910,45 @@
         <v>14</v>
       </c>
       <c r="H32" t="s">
+        <v>141</v>
+      </c>
+      <c r="J32" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="J32" s="2" t="s">
+      <c r="K32" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="K32" s="2" t="s">
-        <v>144</v>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>152</v>
+      </c>
+      <c r="B33">
+        <v>1</v>
+      </c>
+      <c r="C33" t="s">
+        <v>153</v>
+      </c>
+      <c r="D33" t="s">
+        <v>19</v>
+      </c>
+      <c r="E33" t="s">
+        <v>74</v>
+      </c>
+      <c r="F33">
+        <v>2018</v>
+      </c>
+      <c r="G33">
+        <v>2021</v>
+      </c>
+      <c r="H33" t="s">
+        <v>154</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="K33" s="1" t="s">
+        <v>156</v>
       </c>
     </row>
   </sheetData>
@@ -1929,8 +1996,11 @@
     <hyperlink ref="J19" r:id="rId36" display="http://www.linkedin.com/in/sam-durston-812a35293" xr:uid="{41EA5EAB-1092-4025-88C2-6B68516F645F}"/>
     <hyperlink ref="J32" r:id="rId37" xr:uid="{73AD8C54-4705-40A9-9643-92FEFA8BB733}"/>
     <hyperlink ref="K32" r:id="rId38" xr:uid="{5B5AAAAF-F891-4B3C-B316-A8C75688726E}"/>
+    <hyperlink ref="J9" r:id="rId39" display="https://eur01.safelinks.protection.outlook.com/?url=https%3A%2F%2Fwww.linkedin.com%2Fin%2Famber-cowans%2F&amp;data=05%7C02%7Ccss6%40st-andrews.ac.uk%7C7460b5026881483372d408dea14a08be%7Cf85626cb0da849d3aa5864ef678ef01a%7C0%7C0%7C639125536507453985%7CUnknown%7CTWFpbGZsb3d8eyJFbXB0eU1hcGkiOnRydWUsIlYiOiIwLjAuMDAwMCIsIlAiOiJXaW4zMiIsIkFOIjoiTWFpbCIsIldUIjoyfQ%3D%3D%7C0%7C%7C%7C&amp;sdata=owOoj%2BX6dIIVqmzvbwk6odnzWsn5S7FKUDMNke8%2FbQY%3D&amp;reserved=0" xr:uid="{0D7407ED-CA39-44E4-B0C1-181859B0D9F1}"/>
+    <hyperlink ref="I33" r:id="rId40" xr:uid="{550E047B-3A74-4289-80F7-152FE2CC96ED}"/>
+    <hyperlink ref="K33" r:id="rId41" display="https://eur01.safelinks.protection.outlook.com/?url=https%3A%2F%2Fwww.researchgate.net%2Fprofile%2FGoncalo-Curveira-Santos&amp;data=05%7C02%7Ccss6%40st-andrews.ac.uk%7Caa22359e757243cb924208dea2149d24%7Cf85626cb0da849d3aa5864ef678ef01a%7C0%7C0%7C639126406591585183%7CUnknown%7CTWFpbGZsb3d8eyJFbXB0eU1hcGkiOnRydWUsIlYiOiIwLjAuMDAwMCIsIlAiOiJXaW4zMiIsIkFOIjoiTWFpbCIsIldUIjoyfQ%3D%3D%7C0%7C%7C%7C&amp;sdata=dsATszQozywwp1XZVpUIKc8TxsgIEYThxM2mbt5scZM%3D&amp;reserved=0" xr:uid="{9A9CC0B6-BF43-41EA-9520-993C8DB284A6}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId39"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId42"/>
 </worksheet>
 </file>
</xml_diff>